<commit_message>
Mais detalhes: rótulo acima do produto vira 'Plano de internet para sua casa'
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo-ofertas-TEMPLATE.xlsx
+++ b/catalogo-ofertas-TEMPLATE.xlsx
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Plano Claro pós-pago</t>
+          <t>Plano de internet para sua casa</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Plano Claro pós-pago</t>
+          <t>Plano de internet para sua casa</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Plano Claro pós-pago</t>
+          <t>Plano de internet para sua casa</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Mais detalhes: rótulo acima do produto vira 'Plano Claro Fibra'
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo-ofertas-TEMPLATE.xlsx
+++ b/catalogo-ofertas-TEMPLATE.xlsx
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Plano de internet para sua casa</t>
+          <t>Plano Claro Fibra</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Plano de internet para sua casa</t>
+          <t>Plano Claro Fibra</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Plano de internet para sua casa</t>
+          <t>Plano Claro Fibra</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">

</xml_diff>